<commit_message>
feat: add configurable area field to career list sidebar
Add `area` column support to update_career_list so each career can
display its own sub-area label (row 2 of Tabla 8) instead of the
hardcoded template value. Update ejemplo.xlsx with area and separador columns.
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -425,37 +425,47 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>carrera</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>segmento</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>modalidad</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>pain</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>hallazgo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>accion</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>nivel</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>separador</t>
         </is>
       </c>
     </row>
@@ -467,37 +477,47 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Ingenieria</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Ing. Electrónica</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Pagos - Problemas económicos. (2) Perdió trabajo</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>La empresa redujo personal por problemas económicos.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>No aplica.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -509,37 +529,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Ingenieria</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Ing. Electrónica</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Trámites - Fechas de matrícula. (1) Desconocía fecha</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>El alumno se quedó incomunicado al perder su celular.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>No aplica.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -551,37 +581,47 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Ingenieria</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Ing. Electrónica</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Familia - Carrera no disponible. (1) Quiere Educación</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Quiere estudiar Educación Secundaria pero la UTP no la tiene.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>No aplica.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -593,37 +633,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Ingenieria</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Ing. Electrónica</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Asesor comercial - Retiro no atendido. (1)</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Solicitó RPL y no fue atendida.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Validar caso / revisar proceso comercial.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -635,37 +685,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Ingenieria</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Ing. Electrónica</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Cursos - Cursos 24/7. (1) Dificultad para entrar</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Es complicado ingresar a UTP+class para los cursos 24/7.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Revisar contacto en campaña de Bienvenida.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -677,37 +737,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Pagos - Deuda previa. (1)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Generó deuda y no puede seguir pagando.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Derivar a bienestar.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>
@@ -719,37 +789,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Medicina</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Nuevos</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Asesor - Sin seguimiento. (2)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Nunca recibió llamada del asesor asignado.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Auditar gestión del asesor.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>transversal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: agrupar carreras por sección en la barra lateral
- nueva hoja Excel `secciones` (seccion|carrera) como fuente de verdad
- read_secciones + read_excel devuelve (datos, metadata, secciones)
- update_career_list reescrito: menú de secciones dinámico y lista de
  carreras de la sección activa, con sección y carrera resaltadas
- set_cell con formato opcional + nuevo set_cell_lines multi-párrafo
- validaciones en la UI y documentación (README, CLAUDE.md)
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="datos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="secciones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1024,4 +1025,186 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>seccion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>carrera</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Carreras Masivas</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ing. Electrónica</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Carreras Masivas</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ing. de Sistemas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Carreras Masivas</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ing. de Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Carreras Masivas</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Contabilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Carreras Masivas</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Derecho</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Farm. y Bioq</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Enfermería</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Psicología</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ing. Mecánica</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ing. Ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: adaptar barra lateral al template de 4 tarjetas con geometría dinámica
- Tabla 8 ahora son 4 tarjetas de sección (filas 0-3) + lista en fila 4
- la posición de la lista y el offset del grupo se calculan en runtime,
  así el layout se reajusta solo si cambia el template
- la sección activa conserva su tarjeta y se resalta; la flecha apunta
  exacto a la carrera activa
- ejemplo.xlsx: 4 secciones (incluye Carreras Faco de ejemplo)
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -1033,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1111,94 +1111,142 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Medicina</t>
+          <t>Ciencias de la Comunicación</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Farm. y Bioq</t>
+          <t>Comunicación Audiovisual</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Enfermería</t>
+          <t>Diseño Gráfico</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Psicología</t>
+          <t>Periodismo</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Carreras No Masivas</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ing. Automotriz</t>
+          <t>Medicina</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Carreras No Masivas</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ing. Mecánica</t>
+          <t>Farm. y Bioq</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Carreras No Masivas</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ing. Ambiental</t>
+          <t>Enfermería</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Psicología</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Carreras No Masivas</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ing. Mecánica</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ing. Ambiental</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Carreras No Masivas</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Economía</t>
         </is>

</xml_diff>

<commit_message>
feat: expandir las carreras inline bajo la sección activa
- la fila de lista se mueve para quedar justo debajo de la tarjeta de la
  sección activa, empujando las secciones de abajo (antes iba al fondo)
- la posición de la lista y de la flecha se recalculan según dónde quede
- ejemplo.xlsx: Salud = Medicina/Enfermería/Obstetricia
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -1033,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1147,12 +1147,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Carreras Faco</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Periodismo</t>
+          <t>Medicina</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Medicina</t>
+          <t>Enfermería</t>
         </is>
       </c>
     </row>
@@ -1176,31 +1176,31 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Farm. y Bioq</t>
+          <t>Obstetricia</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras No Masivas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enfermería</t>
+          <t>Ing. Automotriz</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras No Masivas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Psicología</t>
+          <t>Ing. Mecánica</t>
         </is>
       </c>
     </row>
@@ -1212,43 +1212,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ing. Automotriz</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Carreras No Masivas</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Ing. Mecánica</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Carreras No Masivas</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
           <t>Ing. Ambiental</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Carreras No Masivas</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Economía</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: ejemplo realista con 4 secciones (masivas, salud, no masivas, faco)
</commit_message>
<xml_diff>
--- a/ejemplo.xlsx
+++ b/ejemplo.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,12 +478,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Ingeniería</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -498,22 +498,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pagos - Problemas económicos. (2) Perdió trabajo</t>
+          <t>Pagos - Problemas económicos. (3) Perdió beca</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>La empresa redujo personal por problemas económicos.</t>
+          <t>El alumno perdió la beca por bajo rendimiento y no puede cubrir la pensión.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>No aplica.</t>
+          <t>Derivar a Servicio de Becas para reevaluación.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>no_accionable</t>
+          <t>profundizar</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -530,12 +530,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Ingeniería</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -550,27 +550,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Trámites - Fechas de matrícula. (1) Desconocía fecha</t>
+          <t>Cursos - Carga académica. (2) Demasiados cursos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>El alumno se quedó incomunicado al perder su celular.</t>
+          <t>Se matriculó en 6 cursos y no logró sostener el ritmo.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>No aplica.</t>
+          <t>Revisar plan de matrícula sugerida para primer ciclo.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>no_accionable</t>
+          <t>profundizar</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>transversal</t>
+          <t>especifico</t>
         </is>
       </c>
     </row>
@@ -582,12 +582,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Ingeniería</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Familia - Carrera no disponible. (1) Quiere Educación</t>
+          <t>Trámites - Plataforma. (1) No accedía al aula</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Quiere estudiar Educación Secundaria pero la UTP no la tiene.</t>
+          <t>Problemas de acceso a UTP+class durante las dos primeras semanas.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Ingeniería</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -654,17 +654,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asesor comercial - Retiro no atendido. (1)</t>
+          <t>Asesor comercial - Sin seguimiento. (2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Solicitó RPL y no fue atendida.</t>
+          <t>No recibió contacto del asesor tras la matrícula.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Validar caso / revisar proceso comercial.</t>
+          <t>Auditar gestión del asesor asignado.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Ingeniería</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -706,17 +706,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cursos - Cursos 24/7. (1) Dificultad para entrar</t>
+          <t>Familia - Mudanza. (1) Se fue de la ciudad</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Es complicado ingresar a UTP+class para los cursos 24/7.</t>
+          <t>La familia se trasladó a provincia por trabajo del padre.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Revisar contacto en campaña de Bienvenida.</t>
+          <t>No aplica.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -758,17 +758,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Pagos - Deuda previa. (1)</t>
+          <t>Pagos - Deuda previa. (2)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Generó deuda y no puede seguir pagando.</t>
+          <t>Generó deuda en el primer ciclo y no pudo regularizar.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Derivar a bienestar.</t>
+          <t>Derivar a Bienestar para plan de pago.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -810,25 +810,493 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asesor - Sin seguimiento. (2)</t>
+          <t>Cursos - Exigencia. (3) Anatomía</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Desaprobó Anatomía y se desmotivó tras el primer parcial.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ofrecer tutoría académica reforzada.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>especifico</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Asesor - Sin seguimiento. (1)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>Nunca recibió llamada del asesor asignado.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Auditar gestión del asesor.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>profundizar</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Familia - Salud. (1) Enfermedad de familiar</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Tuvo que cuidar a un familiar enfermo y abandonó.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No aplica.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>No Masivas</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ingeniería</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Pagos - Problemas económicos. (2)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Ingresos familiares reducidos durante el ciclo.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No aplica.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>No Masivas</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ingeniería</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Vocación - Expectativa de carrera. (2) Esperaba más taller</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Esperaba más prácticas de taller en el primer ciclo.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Revisar comunicación de malla en campaña.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>especifico</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>No Masivas</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ingeniería</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Sede - Distancia. (1) Lejanía del campus</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>El traslado a la sede le tomaba más de 2 horas.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>No aplica.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pagos - Materiales. (2) Costo de insumos</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No pudo cubrir el costo de materiales del curso de taller.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Evaluar kit de insumos en cuotas.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>especifico</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Trámites - Fechas de matrícula. (1)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Desconocía la fecha de matrícula y perdió el ciclo.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Reforzar recordatorios por SMS y correo.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Equipo - Requisitos técnicos. (2) PC insuficiente</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Su equipo no soportaba el software de diseño requerido.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No aplica.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>no_accionable</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Faco</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Asesor comercial - Retiro no atendido. (1)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Solicitó retiro y no fue atendido a tiempo.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Validar caso / revisar proceso comercial.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>profundizar</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>transversal</t>
         </is>
@@ -845,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -908,7 +1376,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -923,7 +1391,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>38.6%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -933,29 +1401,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>62</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Los alumnos desertores tienen un perfil con retraso en pagos.
-El 42% aún tiene deuda.
-26% NSE C y 63% NSE D vs el comparable del segmento.</t>
+          <t>Perfil de desertor con retraso en pagos y alta carga académica.
+El 51% se concentra en el primer ciclo.
+Predomina NSE C y D frente al comparable del segmento.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Muy encima</t>
+          <t>Encima</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1007,8 +1475,8 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Perfil de desertor principalmente por factores económicos.
-Alta incidencia en primer ciclo.</t>
+          <t>Perfil de desertor principalmente por factores económicos y exigencia académica.
+Alta incidencia en cursos de ciencias básicas.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1019,6 +1487,122 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>Mejora</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ing. Automotriz</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>41.0%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>31.4%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Carrera no masiva con muestra reducida.
+Pesa la expectativa de carrera y la distancia a la sede.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Muy encima</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Estable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Nuevos</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>34.2%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>31.4%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Deserción asociada a costos de materiales y requisitos técnicos.
+Foco en habilitar acceso a equipos y software.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Encima</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Empeora</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,7 +1640,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ing. Electrónica</t>
+          <t>Ing. de Sistemas</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1652,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ing. de Sistemas</t>
+          <t>Ing. Industrial</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1664,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ing. de Software</t>
+          <t>Administración</t>
         </is>
       </c>
     </row>
@@ -1111,36 +1695,36 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Carreras Faco</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ciencias de la Comunicación</t>
+          <t>Medicina</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Carreras Faco</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Comunicación Audiovisual</t>
+          <t>Enfermería</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Carreras Faco</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Diseño Gráfico</t>
+          <t>Obstetricia</t>
         </is>
       </c>
     </row>
@@ -1152,31 +1736,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medicina</t>
+          <t>Psicología</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras No Masivas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Enfermería</t>
+          <t>Ing. Automotriz</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Carreras No Masivas</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Obstetricia</t>
+          <t>Ing. Mecánica</t>
         </is>
       </c>
     </row>
@@ -1188,31 +1772,43 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ing. Automotriz</t>
+          <t>Ing. Ambiental</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carreras No Masivas</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ing. Mecánica</t>
+          <t>Ciencias de la Comunicación</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Carreras No Masivas</t>
+          <t>Carreras Faco</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ing. Ambiental</t>
+          <t>Comunicación Audiovisual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Carreras Faco</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
         </is>
       </c>
     </row>

</xml_diff>